<commit_message>
Edit BCIO_External_Imports.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,7 +518,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>has input [RO:0002233]; has output [RO:0002234]; realizes [BFO:0000055]; overlaps [RO:0002131]; output of [RO:0002353]; has input[RO:0002233]; has input [RO:0002233]; causally influenced by [RO:0002559]; causal relation between entities [RO:0002506]; temporally related to [RO:0002222]; realized in [BFO:0000054]; occurs in [BFO:0000066]</t>
+          <t>has input [RO:0002233]; has output [RO:0002234]; realizes [BFO:0000055]; overlaps [RO:0002131]; output of [RO:0002353]; has input[RO:0002233]; has input [RO:0002233]; causally influenced by [RO:0002559]; causal relation between entities [RO:0002506]; temporally related to [RO:0002222]; realized in [BFO:0000054]; occurs in [BFO:0000066]; preceded by [BFO:0000062]; precedes [BFO:0000063]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1123,6 +1123,16 @@
           <t>"GMHO: https://galenos.org.uk/ontologies/GMHO_"</t>
         </is>
       </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Row 20 to BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -1125,11 +1125,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>COB</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/COB.owl</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>process [BFO:0000015]</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>planned process [COB:0000082]</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>

</xml_diff>

<commit_message>
Update Row 20 in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -1135,6 +1135,11 @@
           <t>http://purl.obolibrary.org/obo/COB.owl</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/OBOFoundry/COB/2b7d820f804fc9fa17aba5a21a9ce2f821dc5c83/cob.owl</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>process [BFO:0000015]</t>
@@ -1143,6 +1148,11 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>planned process [COB:0000082]</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>all</t>
         </is>
       </c>
     </row>
@@ -1172,13 +1182,11 @@
           <t xml:space="preserve">organisation [OBI:0000245]; </t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Row 8 in BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -742,14 +742,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>money [OMRSE:00000235]; rehabilitation facility [OMRSE:00000106]; hospice facility [OMRSE:00000104]; household [OMRSE:00000076]; residential facility [OMRSE:00000191]; policy holder role [OMRSE:00000094]; healthcare facility [OMRSE:00000102]; emergency department facility [OMRSE:00000114]; hospital facility [OMRSE:00000063]; school facility [OMRSE:00000064]; facility [OMRSE:00000062]; architectural structure [OMRSE:00000061]; household income [OMRSE:00000929]; government assistance income data item [OMRSE:00000504]</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>insured party role [OMRSE:00000092]</t>
-        </is>
-      </c>
+          <t>insured party role [OMRSE:00000092]; 
+money [OMRSE:00000235]; rehabilitation facility [OMRSE:00000106]; hospice facility [OMRSE:00000104]; household [OMRSE:00000076]; residential facility [OMRSE:00000191]; policy holder role [OMRSE:00000094]; healthcare facility [OMRSE:00000102]; emergency department facility [OMRSE:00000114]; hospital facility [OMRSE:00000063]; school facility [OMRSE:00000064]; facility [OMRSE:00000062]; architectural structure [OMRSE:00000061]; household income [OMRSE:00000929]; government assistance income data item [OMRSE:00000504]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>all</t>

</xml_diff>

<commit_message>
Delete Row 19 from BCIO_External_Imports.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_External_Imports.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -746,7 +746,6 @@
 money [OMRSE:00000235]; rehabilitation facility [OMRSE:00000106]; hospice facility [OMRSE:00000104]; household [OMRSE:00000076]; residential facility [OMRSE:00000191]; policy holder role [OMRSE:00000094]; healthcare facility [OMRSE:00000102]; emergency department facility [OMRSE:00000114]; hospital facility [OMRSE:00000063]; school facility [OMRSE:00000064]; facility [OMRSE:00000062]; architectural structure [OMRSE:00000061]; household income [OMRSE:00000929]; government assistance income data item [OMRSE:00000504]</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>all</t>
@@ -1086,100 +1085,62 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GMHO</t>
+          <t>COB</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/galenos-project/mental-health-ontology/refs/heads/main/gmho.owl</t>
+          <t>http://purl.obolibrary.org/obo/COB.owl</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/galenos-project/mental-health-ontology/407a0e714545acabfc2f54cceed4cab2a50be446/gmho.owl</t>
+          <t>https://raw.githubusercontent.com/OBOFoundry/COB/2b7d820f804fc9fa17aba5a21a9ce2f821dc5c83/cob.owl</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>entity [BFO:0000001]</t>
+          <t>process [BFO:0000015]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-intervention context [GMHO:0000253]; intervention temporal context [GMHO:0000254]; process context [GMHO:0000268]</t>
+          <t>planned process [COB:0000082]</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>all</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>"GMHO: https://galenos.org.uk/ontologies/GMHO_"</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COB</t>
+          <t>OBI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>http://purl.obolibrary.org/obo/COB.owl</t>
+          <t>http://purl.obolibrary.org/obo/obi.owl</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/OBOFoundry/COB/2b7d820f804fc9fa17aba5a21a9ce2f821dc5c83/cob.owl</t>
+          <t>http://purl.obolibrary.org/obo/obi/2025-01-09/obi.owl</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>process [BFO:0000015]</t>
+          <t>material entity [BFO:0000040]</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>planned process [COB:0000082]</t>
+          <t xml:space="preserve">organisation [OBI:0000245]; </t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>OBI</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/obi.owl</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/obi/2025-01-09/obi.owl</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>material entity [BFO:0000040]</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">organisation [OBI:0000245]; </t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
         <is>
           <t>all</t>
         </is>

</xml_diff>